<commit_message>
chore: ignore .allure directory in gitignore and update latest Excel report
</commit_message>
<xml_diff>
--- a/KetQuaKiemThu_Login.xlsx
+++ b/KetQuaKiemThu_Login.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="100">
   <si>
     <t>BÁO CÁO KẾT QUẢ KIỂM THỬ TỰ ĐỘNG - LOGIN TEST</t>
   </si>
@@ -20,7 +20,7 @@
     <t>Hệ thống: Văn phòng điện tử UTC (vanphongdientu.utc.edu.vn)</t>
   </si>
   <si>
-    <t>Mã SV: 6451071069 | Thời gian thực hiện: 08/10/2026 15:36:35</t>
+    <t>Mã SV: 6451071069 | Thời gian thực hiện: 08/10/2026 15:39:55</t>
   </si>
   <si>
     <t>STT / Mã TC</t>
@@ -59,7 +59,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>15:35:57</t>
+    <t>15:38:39</t>
   </si>
   <si>
     <t>TC2</t>
@@ -74,7 +74,7 @@
     <t>Bạn chưa nhập mật khẩu</t>
   </si>
   <si>
-    <t>15:36:00</t>
+    <t>15:38:46</t>
   </si>
   <si>
     <t>TC3</t>
@@ -86,13 +86,13 @@
     <t>username: 'huongnt', password: 'utc@235'</t>
   </si>
   <si>
-    <t>Tài khoản không đúng</t>
+    <t>Tài khoản không đúng (hoặc Tài khoản hoặc mật khẩu không đúng.)</t>
   </si>
   <si>
     <t>Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>15:36:03</t>
+    <t>15:38:51</t>
   </si>
   <si>
     <t>TC4</t>
@@ -104,7 +104,7 @@
     <t>username: 'huongthunguyen', password: '123456@utc'</t>
   </si>
   <si>
-    <t>15:36:06</t>
+    <t>15:38:56</t>
   </si>
   <si>
     <t>TC5</t>
@@ -116,13 +116,13 @@
     <t>username: 'huongnt', password: '123456@utc', rememberMe: true</t>
   </si>
   <si>
-    <t>Đưa vào trang chủ (ghi nhớ phiên)</t>
-  </si>
-  <si>
-    <t>Gửi request đăng nhập kèm ghi nhớ thành công</t>
-  </si>
-  <si>
-    <t>15:36:08</t>
+    <t>Tích chọn ghi nhớ thành công và gửi request đăng nhập</t>
+  </si>
+  <si>
+    <t>Đã tích chọn 'Giữ tôi luôn đăng nhập' và submit form thành công</t>
+  </si>
+  <si>
+    <t>15:39:01</t>
   </si>
   <si>
     <t>TC6</t>
@@ -134,13 +134,13 @@
     <t>username: 'huongnt', password: '123456@utc', rememberMe: false</t>
   </si>
   <si>
-    <t>Đưa vào trang chủ (không lưu phiên)</t>
-  </si>
-  <si>
-    <t>Gửi request đăng nhập không lưu phiên thành công</t>
-  </si>
-  <si>
-    <t>15:36:11</t>
+    <t>Không tích chọn ghi nhớ và gửi request đăng nhập bình thường</t>
+  </si>
+  <si>
+    <t>Đã thực hiện gửi request đăng nhập không lưu phiên</t>
+  </si>
+  <si>
+    <t>15:39:06</t>
   </si>
   <si>
     <t>TC7</t>
@@ -152,10 +152,10 @@
     <t>username: '', password: ''</t>
   </si>
   <si>
-    <t>Bạn chưa nhập tên đăng nhập và mật khẩu</t>
-  </si>
-  <si>
-    <t>15:36:13</t>
+    <t>Bạn chưa nhập tên đăng nhập (hoặc Bạn chưa nhập tên đăng nhập và mật khẩu)</t>
+  </si>
+  <si>
+    <t>15:39:10</t>
   </si>
   <si>
     <t>TC8</t>
@@ -167,10 +167,10 @@
     <t>username: '' OR '1'='1', password: '123'</t>
   </si>
   <si>
-    <t>Tài khoản không đúng (chặn SQLi)</t>
-  </si>
-  <si>
-    <t>15:36:16</t>
+    <t>Hệ thống chặn truy cập, báo lỗi Tài khoản hoặc mật khẩu không đúng.</t>
+  </si>
+  <si>
+    <t>15:39:15</t>
   </si>
   <si>
     <t>TC9</t>
@@ -182,7 +182,7 @@
     <t>username: 'admin\' --', password: 'password123'</t>
   </si>
   <si>
-    <t>15:36:19</t>
+    <t>15:39:20</t>
   </si>
   <si>
     <t>TC10</t>
@@ -194,97 +194,100 @@
     <t>username: '  huongnt  ', password: '123456@utc'</t>
   </si>
   <si>
-    <t>Hệ thống trim khoảng trắng hoặc xử lý an toàn</t>
+    <t>Hệ thống tự động trim khoảng trắng hoặc xử lý an toàn</t>
+  </si>
+  <si>
+    <t>Hệ thống đã nhận diện và xử lý request chứa khoảng trắng: Tài khoản hoặc mật khẩu không đúng.</t>
+  </si>
+  <si>
+    <t>15:39:26</t>
+  </si>
+  <si>
+    <t>TC11</t>
+  </si>
+  <si>
+    <t>Nhập tên đăng nhập phân biệt chữ hoa, chữ thường</t>
+  </si>
+  <si>
+    <t>username: 'HuongNT', password: '123456@utc'</t>
+  </si>
+  <si>
+    <t>Hệ thống xác thực tên đăng nhập chữ hoa/chữ thường</t>
+  </si>
+  <si>
+    <t>Phản hồi hệ thống khi nhập username chữ hoa: Tài khoản hoặc mật khẩu không đúng.</t>
+  </si>
+  <si>
+    <t>15:39:31</t>
+  </si>
+  <si>
+    <t>TC12</t>
+  </si>
+  <si>
+    <t>Nhập mật khẩu có phân biệt chữ hoa, chữ thường</t>
+  </si>
+  <si>
+    <t>username: 'huongnt', password: '123456@UTC'</t>
+  </si>
+  <si>
+    <t>Báo lỗi Tài khoản hoặc mật khẩu không đúng.</t>
+  </si>
+  <si>
+    <t>15:39:36</t>
+  </si>
+  <si>
+    <t>TC13</t>
+  </si>
+  <si>
+    <t>Kiểm thử ẩn/hiện ký tự ở ô mật khẩu</t>
+  </si>
+  <si>
+    <t>password: 'MySecretPassword123'</t>
+  </si>
+  <si>
+    <t>Ô mật khẩu có thuộc tính type='password' để ẩn ký tự dạng dấu chấm/sao</t>
+  </si>
+  <si>
+    <t>Thuộc tính type của ô mật khẩu là: password</t>
+  </si>
+  <si>
+    <t>15:39:39</t>
+  </si>
+  <si>
+    <t>TC14</t>
+  </si>
+  <si>
+    <t>Kiểm thử tấn công XSS ở ô username</t>
+  </si>
+  <si>
+    <t>username: '&lt;script&gt;alert(\'XSS\')&lt;/script&gt;', password: 'password123'</t>
+  </si>
+  <si>
+    <t>Hệ thống không thực thi script, không bật alert XSS, báo lỗi an toàn</t>
+  </si>
+  <si>
+    <t>Hệ thống chặn script thành công: Tài khoản hoặc mật khẩu không đúng.</t>
+  </si>
+  <si>
+    <t>15:39:45</t>
+  </si>
+  <si>
+    <t>TC15</t>
+  </si>
+  <si>
+    <t>Nhập chuỗi ký tự quá dài vào ô username và password</t>
+  </si>
+  <si>
+    <t>username: 255 ký tự, password: 255 ký tự</t>
+  </si>
+  <si>
+    <t>Hệ thống xử lý chuỗi dài an toàn, không bị lỗi máy chủ (500)</t>
   </si>
   <si>
     <t>Hệ thống xử lý an toàn: Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>15:36:22</t>
-  </si>
-  <si>
-    <t>TC11</t>
-  </si>
-  <si>
-    <t>Nhập tên đăng nhập phân biệt chữ hoa, chữ thường</t>
-  </si>
-  <si>
-    <t>username: 'HuongNT', password: '123456@utc'</t>
-  </si>
-  <si>
-    <t>Hệ thống xác thực tên người dùng chữ hoa/thường</t>
-  </si>
-  <si>
-    <t>Phản hồi hệ thống: Tài khoản hoặc mật khẩu không đúng.</t>
-  </si>
-  <si>
-    <t>15:36:25</t>
-  </si>
-  <si>
-    <t>TC12</t>
-  </si>
-  <si>
-    <t>Nhập mật khẩu có phân biệt chữ hoa, chữ thường</t>
-  </si>
-  <si>
-    <t>username: 'huongnt', password: '123456@UTC'</t>
-  </si>
-  <si>
-    <t>15:36:27</t>
-  </si>
-  <si>
-    <t>TC13</t>
-  </si>
-  <si>
-    <t>Kiểm thử ẩn/hiện ký tự ở ô mật khẩu</t>
-  </si>
-  <si>
-    <t>password: 'SecretPass123'</t>
-  </si>
-  <si>
-    <t>Mật khẩu ẩn dưới dạng dấu chấm (type='password')</t>
-  </si>
-  <si>
-    <t>Thuộc tính type của ô pass: password</t>
-  </si>
-  <si>
-    <t>15:36:28</t>
-  </si>
-  <si>
-    <t>TC14</t>
-  </si>
-  <si>
-    <t>Kiểm thử tấn công XSS ở ô username</t>
-  </si>
-  <si>
-    <t>username: '&lt;script&gt;alert(\'XSS\')&lt;/script&gt;', password: '123456'</t>
-  </si>
-  <si>
-    <t>Không thực thi mã script, không bật alert</t>
-  </si>
-  <si>
-    <t>Không bật alert, phản hồi an toàn: Tài khoản hoặc mật khẩu không đúng.</t>
-  </si>
-  <si>
-    <t>15:36:31</t>
-  </si>
-  <si>
-    <t>TC15</t>
-  </si>
-  <si>
-    <t>Nhập chuỗi ký tự quá dài vào ô username và password</t>
-  </si>
-  <si>
-    <t>username: 255 ký tự, password: 255 ký tự</t>
-  </si>
-  <si>
-    <t>Hệ thống xử lý an toàn, không crash server (500)</t>
-  </si>
-  <si>
-    <t>Phản hồi hệ thống an toàn: Tài khoản hoặc mật khẩu không đúng.</t>
-  </si>
-  <si>
-    <t>15:36:33</t>
+    <t>15:39:50</t>
   </si>
   <si>
     <t>TC16</t>
@@ -293,16 +296,16 @@
     <t>Kiểm thử tính năng Paste vào ô password</t>
   </si>
   <si>
-    <t>Dán chuỗi: '123456@utc'</t>
-  </si>
-  <si>
-    <t>Chuỗi mật khẩu được dán thành công</t>
-  </si>
-  <si>
-    <t>Giá trị ô pass sau khi dán: 123456@utc</t>
-  </si>
-  <si>
-    <t>15:36:34</t>
+    <t>Dán (Ctrl + V) chuỗi: 123456@utc</t>
+  </si>
+  <si>
+    <t>Chuỗi mật khẩu được dán thành công vào ô password</t>
+  </si>
+  <si>
+    <t>Giá trị sau khi dán vào ô mật khẩu: 123456@utc</t>
+  </si>
+  <si>
+    <t>15:39:55</t>
   </si>
   <si>
     <t>TỔNG SỐ TEST CASE: 16</t>
@@ -459,9 +462,9 @@
   <cols>
     <col min="1" max="1" width="57.01953125" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="55.62890625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="59.87890625" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="47.4296875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="63.921875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="60.40234375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="69.9921875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="84.01171875" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="15.625" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="18.08203125" customWidth="true" bestFit="true"/>
   </cols>
@@ -699,7 +702,7 @@
         <v>55</v>
       </c>
       <c r="D14" t="s" s="2">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="E14" t="s" s="2">
         <v>25</v>
@@ -768,7 +771,7 @@
         <v>71</v>
       </c>
       <c r="D17" t="s" s="2">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="E17" t="s" s="2">
         <v>25</v>
@@ -777,109 +780,109 @@
         <v>14</v>
       </c>
       <c r="G17" t="s" s="3">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" ht="22.0" customHeight="true">
       <c r="A18" t="s" s="3">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C18" t="s" s="2">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D18" t="s" s="2">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E18" t="s" s="2">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F18" t="s" s="4">
         <v>14</v>
       </c>
       <c r="G18" t="s" s="3">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19" ht="22.0" customHeight="true">
       <c r="A19" t="s" s="3">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C19" t="s" s="2">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D19" t="s" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E19" t="s" s="2">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F19" t="s" s="4">
         <v>14</v>
       </c>
       <c r="G19" t="s" s="3">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" ht="22.0" customHeight="true">
       <c r="A20" t="s" s="3">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C20" t="s" s="2">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D20" t="s" s="2">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E20" t="s" s="2">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F20" t="s" s="4">
         <v>14</v>
       </c>
       <c r="G20" t="s" s="3">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" ht="22.0" customHeight="true">
       <c r="A21" t="s" s="3">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C21" t="s" s="2">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D21" t="s" s="2">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E21" t="s" s="2">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F21" t="s" s="4">
         <v>14</v>
       </c>
       <c r="G21" t="s" s="3">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="s" s="6">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="s" s="6">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: align project architecture with lecture slide 48 and apply Explicit Wait standard
</commit_message>
<xml_diff>
--- a/KetQuaKiemThu_Login.xlsx
+++ b/KetQuaKiemThu_Login.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="98">
   <si>
     <t>BÁO CÁO KẾT QUẢ KIỂM THỬ TỰ ĐỘNG - LOGIN TEST</t>
   </si>
@@ -20,7 +20,7 @@
     <t>Hệ thống: Văn phòng điện tử UTC (vanphongdientu.utc.edu.vn)</t>
   </si>
   <si>
-    <t>Mã SV: 6451071069 | Thời gian thực hiện: 08/10/2026 15:39:55</t>
+    <t>Mã SV: 6451071069 | Thời gian thực hiện: 08/10/2026 16:26:23</t>
   </si>
   <si>
     <t>STT / Mã TC</t>
@@ -59,7 +59,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>15:38:39</t>
+    <t>16:25:34</t>
   </si>
   <si>
     <t>TC2</t>
@@ -74,7 +74,7 @@
     <t>Bạn chưa nhập mật khẩu</t>
   </si>
   <si>
-    <t>15:38:46</t>
+    <t>16:25:37</t>
   </si>
   <si>
     <t>TC3</t>
@@ -92,7 +92,7 @@
     <t>Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>15:38:51</t>
+    <t>16:25:40</t>
   </si>
   <si>
     <t>TC4</t>
@@ -104,7 +104,7 @@
     <t>username: 'huongthunguyen', password: '123456@utc'</t>
   </si>
   <si>
-    <t>15:38:56</t>
+    <t>16:25:43</t>
   </si>
   <si>
     <t>TC5</t>
@@ -119,10 +119,10 @@
     <t>Tích chọn ghi nhớ thành công và gửi request đăng nhập</t>
   </si>
   <si>
-    <t>Đã tích chọn 'Giữ tôi luôn đăng nhập' và submit form thành công</t>
-  </si>
-  <si>
-    <t>15:39:01</t>
+    <t>Đã tích chọn 'Giữ tôi luôn đăng nhập' và gửi request thành công</t>
+  </si>
+  <si>
+    <t>16:25:46</t>
   </si>
   <si>
     <t>TC6</t>
@@ -140,7 +140,7 @@
     <t>Đã thực hiện gửi request đăng nhập không lưu phiên</t>
   </si>
   <si>
-    <t>15:39:06</t>
+    <t>16:25:49</t>
   </si>
   <si>
     <t>TC7</t>
@@ -152,10 +152,7 @@
     <t>username: '', password: ''</t>
   </si>
   <si>
-    <t>Bạn chưa nhập tên đăng nhập (hoặc Bạn chưa nhập tên đăng nhập và mật khẩu)</t>
-  </si>
-  <si>
-    <t>15:39:10</t>
+    <t>16:25:52</t>
   </si>
   <si>
     <t>TC8</t>
@@ -170,7 +167,7 @@
     <t>Hệ thống chặn truy cập, báo lỗi Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>15:39:15</t>
+    <t>16:25:56</t>
   </si>
   <si>
     <t>TC9</t>
@@ -182,7 +179,7 @@
     <t>username: 'admin\' --', password: 'password123'</t>
   </si>
   <si>
-    <t>15:39:20</t>
+    <t>16:26:01</t>
   </si>
   <si>
     <t>TC10</t>
@@ -197,10 +194,10 @@
     <t>Hệ thống tự động trim khoảng trắng hoặc xử lý an toàn</t>
   </si>
   <si>
-    <t>Hệ thống đã nhận diện và xử lý request chứa khoảng trắng: Tài khoản hoặc mật khẩu không đúng.</t>
-  </si>
-  <si>
-    <t>15:39:26</t>
+    <t>Hệ thống xử lý an toàn: Tài khoản hoặc mật khẩu không đúng.</t>
+  </si>
+  <si>
+    <t>16:26:05</t>
   </si>
   <si>
     <t>TC11</t>
@@ -215,10 +212,10 @@
     <t>Hệ thống xác thực tên đăng nhập chữ hoa/chữ thường</t>
   </si>
   <si>
-    <t>Phản hồi hệ thống khi nhập username chữ hoa: Tài khoản hoặc mật khẩu không đúng.</t>
-  </si>
-  <si>
-    <t>15:39:31</t>
+    <t>Phản hồi hệ thống: Tài khoản hoặc mật khẩu không đúng.</t>
+  </si>
+  <si>
+    <t>16:26:08</t>
   </si>
   <si>
     <t>TC12</t>
@@ -233,7 +230,7 @@
     <t>Báo lỗi Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>15:39:36</t>
+    <t>16:26:11</t>
   </si>
   <si>
     <t>TC13</t>
@@ -251,7 +248,7 @@
     <t>Thuộc tính type của ô mật khẩu là: password</t>
   </si>
   <si>
-    <t>15:39:39</t>
+    <t>16:26:13</t>
   </si>
   <si>
     <t>TC14</t>
@@ -269,7 +266,7 @@
     <t>Hệ thống chặn script thành công: Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>15:39:45</t>
+    <t>16:26:16</t>
   </si>
   <si>
     <t>TC15</t>
@@ -284,10 +281,7 @@
     <t>Hệ thống xử lý chuỗi dài an toàn, không bị lỗi máy chủ (500)</t>
   </si>
   <si>
-    <t>Hệ thống xử lý an toàn: Tài khoản hoặc mật khẩu không đúng.</t>
-  </si>
-  <si>
-    <t>15:39:50</t>
+    <t>16:26:19</t>
   </si>
   <si>
     <t>TC16</t>
@@ -305,7 +299,7 @@
     <t>Giá trị sau khi dán vào ô mật khẩu: 123456@utc</t>
   </si>
   <si>
-    <t>15:39:55</t>
+    <t>16:26:22</t>
   </si>
   <si>
     <t>TỔNG SỐ TEST CASE: 16</t>
@@ -463,8 +457,8 @@
     <col min="1" max="1" width="57.01953125" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="55.62890625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="60.40234375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="69.9921875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="84.01171875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="65.18359375" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="63.0625" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="15.625" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="18.08203125" customWidth="true" bestFit="true"/>
   </cols>
@@ -656,7 +650,7 @@
         <v>45</v>
       </c>
       <c r="D12" t="s" s="2">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="E12" t="s" s="2">
         <v>13</v>
@@ -665,21 +659,21 @@
         <v>14</v>
       </c>
       <c r="G12" t="s" s="3">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" ht="22.0" customHeight="true">
       <c r="A13" t="s" s="3">
+        <v>47</v>
+      </c>
+      <c r="B13" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="B13" t="s" s="2">
+      <c r="C13" t="s" s="2">
         <v>49</v>
       </c>
-      <c r="C13" t="s" s="2">
+      <c r="D13" t="s" s="2">
         <v>50</v>
-      </c>
-      <c r="D13" t="s" s="2">
-        <v>51</v>
       </c>
       <c r="E13" t="s" s="2">
         <v>25</v>
@@ -688,21 +682,21 @@
         <v>14</v>
       </c>
       <c r="G13" t="s" s="3">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" ht="22.0" customHeight="true">
       <c r="A14" t="s" s="3">
+        <v>52</v>
+      </c>
+      <c r="B14" t="s" s="2">
         <v>53</v>
       </c>
-      <c r="B14" t="s" s="2">
+      <c r="C14" t="s" s="2">
         <v>54</v>
       </c>
-      <c r="C14" t="s" s="2">
-        <v>55</v>
-      </c>
       <c r="D14" t="s" s="2">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E14" t="s" s="2">
         <v>25</v>
@@ -711,67 +705,67 @@
         <v>14</v>
       </c>
       <c r="G14" t="s" s="3">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" ht="22.0" customHeight="true">
       <c r="A15" t="s" s="3">
+        <v>56</v>
+      </c>
+      <c r="B15" t="s" s="2">
         <v>57</v>
       </c>
-      <c r="B15" t="s" s="2">
+      <c r="C15" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="C15" t="s" s="2">
+      <c r="D15" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="D15" t="s" s="2">
+      <c r="E15" t="s" s="2">
         <v>60</v>
       </c>
-      <c r="E15" t="s" s="2">
+      <c r="F15" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="G15" t="s" s="3">
         <v>61</v>
-      </c>
-      <c r="F15" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="G15" t="s" s="3">
-        <v>62</v>
       </c>
     </row>
     <row r="16" ht="22.0" customHeight="true">
       <c r="A16" t="s" s="3">
+        <v>62</v>
+      </c>
+      <c r="B16" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="B16" t="s" s="2">
+      <c r="C16" t="s" s="2">
         <v>64</v>
       </c>
-      <c r="C16" t="s" s="2">
+      <c r="D16" t="s" s="2">
         <v>65</v>
       </c>
-      <c r="D16" t="s" s="2">
+      <c r="E16" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="E16" t="s" s="2">
+      <c r="F16" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="G16" t="s" s="3">
         <v>67</v>
-      </c>
-      <c r="F16" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="G16" t="s" s="3">
-        <v>68</v>
       </c>
     </row>
     <row r="17" ht="22.0" customHeight="true">
       <c r="A17" t="s" s="3">
+        <v>68</v>
+      </c>
+      <c r="B17" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="B17" t="s" s="2">
+      <c r="C17" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="C17" t="s" s="2">
+      <c r="D17" t="s" s="2">
         <v>71</v>
-      </c>
-      <c r="D17" t="s" s="2">
-        <v>72</v>
       </c>
       <c r="E17" t="s" s="2">
         <v>25</v>
@@ -780,109 +774,109 @@
         <v>14</v>
       </c>
       <c r="G17" t="s" s="3">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" ht="22.0" customHeight="true">
       <c r="A18" t="s" s="3">
+        <v>73</v>
+      </c>
+      <c r="B18" t="s" s="2">
         <v>74</v>
       </c>
-      <c r="B18" t="s" s="2">
+      <c r="C18" t="s" s="2">
         <v>75</v>
       </c>
-      <c r="C18" t="s" s="2">
+      <c r="D18" t="s" s="2">
         <v>76</v>
       </c>
-      <c r="D18" t="s" s="2">
+      <c r="E18" t="s" s="2">
         <v>77</v>
       </c>
-      <c r="E18" t="s" s="2">
+      <c r="F18" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="G18" t="s" s="3">
         <v>78</v>
-      </c>
-      <c r="F18" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="G18" t="s" s="3">
-        <v>79</v>
       </c>
     </row>
     <row r="19" ht="22.0" customHeight="true">
       <c r="A19" t="s" s="3">
+        <v>79</v>
+      </c>
+      <c r="B19" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="B19" t="s" s="2">
+      <c r="C19" t="s" s="2">
         <v>81</v>
       </c>
-      <c r="C19" t="s" s="2">
+      <c r="D19" t="s" s="2">
         <v>82</v>
       </c>
-      <c r="D19" t="s" s="2">
+      <c r="E19" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="E19" t="s" s="2">
+      <c r="F19" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="G19" t="s" s="3">
         <v>84</v>
-      </c>
-      <c r="F19" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="G19" t="s" s="3">
-        <v>85</v>
       </c>
     </row>
     <row r="20" ht="22.0" customHeight="true">
       <c r="A20" t="s" s="3">
+        <v>85</v>
+      </c>
+      <c r="B20" t="s" s="2">
         <v>86</v>
       </c>
-      <c r="B20" t="s" s="2">
+      <c r="C20" t="s" s="2">
         <v>87</v>
       </c>
-      <c r="C20" t="s" s="2">
+      <c r="D20" t="s" s="2">
         <v>88</v>
       </c>
-      <c r="D20" t="s" s="2">
+      <c r="E20" t="s" s="2">
+        <v>60</v>
+      </c>
+      <c r="F20" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="G20" t="s" s="3">
         <v>89</v>
-      </c>
-      <c r="E20" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="F20" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="G20" t="s" s="3">
-        <v>91</v>
       </c>
     </row>
     <row r="21" ht="22.0" customHeight="true">
       <c r="A21" t="s" s="3">
+        <v>90</v>
+      </c>
+      <c r="B21" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="C21" t="s" s="2">
         <v>92</v>
       </c>
-      <c r="B21" t="s" s="2">
+      <c r="D21" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="C21" t="s" s="2">
+      <c r="E21" t="s" s="2">
         <v>94</v>
       </c>
-      <c r="D21" t="s" s="2">
+      <c r="F21" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="G21" t="s" s="3">
         <v>95</v>
-      </c>
-      <c r="E21" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="F21" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="G21" t="s" s="3">
-        <v>97</v>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="s" s="6">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="s" s="6">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: update latest Excel test execution report with cleaned results
</commit_message>
<xml_diff>
--- a/KetQuaKiemThu_Login.xlsx
+++ b/KetQuaKiemThu_Login.xlsx
@@ -20,7 +20,7 @@
     <t>Hệ thống: Văn phòng điện tử UTC (vanphongdientu.utc.edu.vn)</t>
   </si>
   <si>
-    <t>Mã SV: 6451071069 | Thời gian thực hiện: 08/10/2026 16:26:23</t>
+    <t>Mã SV: 6451071069 | Thời gian thực hiện: 08/10/2026 16:31:17</t>
   </si>
   <si>
     <t>STT / Mã TC</t>
@@ -59,7 +59,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>16:25:34</t>
+    <t>16:30:36</t>
   </si>
   <si>
     <t>TC2</t>
@@ -74,7 +74,7 @@
     <t>Bạn chưa nhập mật khẩu</t>
   </si>
   <si>
-    <t>16:25:37</t>
+    <t>16:30:39</t>
   </si>
   <si>
     <t>TC3</t>
@@ -92,7 +92,7 @@
     <t>Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>16:25:40</t>
+    <t>16:30:42</t>
   </si>
   <si>
     <t>TC4</t>
@@ -104,7 +104,7 @@
     <t>username: 'huongthunguyen', password: '123456@utc'</t>
   </si>
   <si>
-    <t>16:25:43</t>
+    <t>16:30:45</t>
   </si>
   <si>
     <t>TC5</t>
@@ -122,7 +122,7 @@
     <t>Đã tích chọn 'Giữ tôi luôn đăng nhập' và gửi request thành công</t>
   </si>
   <si>
-    <t>16:25:46</t>
+    <t>16:30:48</t>
   </si>
   <si>
     <t>TC6</t>
@@ -140,7 +140,7 @@
     <t>Đã thực hiện gửi request đăng nhập không lưu phiên</t>
   </si>
   <si>
-    <t>16:25:49</t>
+    <t>16:30:50</t>
   </si>
   <si>
     <t>TC7</t>
@@ -152,7 +152,7 @@
     <t>username: '', password: ''</t>
   </si>
   <si>
-    <t>16:25:52</t>
+    <t>16:30:53</t>
   </si>
   <si>
     <t>TC8</t>
@@ -167,7 +167,7 @@
     <t>Hệ thống chặn truy cập, báo lỗi Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>16:25:56</t>
+    <t>16:30:56</t>
   </si>
   <si>
     <t>TC9</t>
@@ -179,7 +179,7 @@
     <t>username: 'admin\' --', password: 'password123'</t>
   </si>
   <si>
-    <t>16:26:01</t>
+    <t>16:30:58</t>
   </si>
   <si>
     <t>TC10</t>
@@ -197,7 +197,7 @@
     <t>Hệ thống xử lý an toàn: Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>16:26:05</t>
+    <t>16:31:01</t>
   </si>
   <si>
     <t>TC11</t>
@@ -215,7 +215,7 @@
     <t>Phản hồi hệ thống: Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>16:26:08</t>
+    <t>16:31:04</t>
   </si>
   <si>
     <t>TC12</t>
@@ -230,7 +230,7 @@
     <t>Báo lỗi Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>16:26:11</t>
+    <t>16:31:06</t>
   </si>
   <si>
     <t>TC13</t>
@@ -248,7 +248,7 @@
     <t>Thuộc tính type của ô mật khẩu là: password</t>
   </si>
   <si>
-    <t>16:26:13</t>
+    <t>16:31:09</t>
   </si>
   <si>
     <t>TC14</t>
@@ -266,7 +266,7 @@
     <t>Hệ thống chặn script thành công: Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>16:26:16</t>
+    <t>16:31:11</t>
   </si>
   <si>
     <t>TC15</t>
@@ -281,7 +281,7 @@
     <t>Hệ thống xử lý chuỗi dài an toàn, không bị lỗi máy chủ (500)</t>
   </si>
   <si>
-    <t>16:26:19</t>
+    <t>16:31:14</t>
   </si>
   <si>
     <t>TC16</t>
@@ -299,7 +299,7 @@
     <t>Giá trị sau khi dán vào ô mật khẩu: 123456@utc</t>
   </si>
   <si>
-    <t>16:26:22</t>
+    <t>16:31:16</t>
   </si>
   <si>
     <t>TỔNG SỐ TEST CASE: 16</t>

</xml_diff>

<commit_message>
docs: remove redundant comments and clean up documentation
</commit_message>
<xml_diff>
--- a/KetQuaKiemThu_Login.xlsx
+++ b/KetQuaKiemThu_Login.xlsx
@@ -20,7 +20,7 @@
     <t>Hệ thống: Văn phòng điện tử UTC (vanphongdientu.utc.edu.vn)</t>
   </si>
   <si>
-    <t>Mã SV: 6451071069 | Thời gian thực hiện: 08/10/2026 16:31:17</t>
+    <t>Mã SV: 6451071069 | Thời gian thực hiện: 08/10/2026 16:48:47</t>
   </si>
   <si>
     <t>STT / Mã TC</t>
@@ -59,7 +59,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>16:30:36</t>
+    <t>16:47:51</t>
   </si>
   <si>
     <t>TC2</t>
@@ -74,7 +74,7 @@
     <t>Bạn chưa nhập mật khẩu</t>
   </si>
   <si>
-    <t>16:30:39</t>
+    <t>16:47:56</t>
   </si>
   <si>
     <t>TC3</t>
@@ -92,7 +92,7 @@
     <t>Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>16:30:42</t>
+    <t>16:47:59</t>
   </si>
   <si>
     <t>TC4</t>
@@ -104,7 +104,7 @@
     <t>username: 'huongthunguyen', password: '123456@utc'</t>
   </si>
   <si>
-    <t>16:30:45</t>
+    <t>16:48:01</t>
   </si>
   <si>
     <t>TC5</t>
@@ -122,7 +122,7 @@
     <t>Đã tích chọn 'Giữ tôi luôn đăng nhập' và gửi request thành công</t>
   </si>
   <si>
-    <t>16:30:48</t>
+    <t>16:48:09</t>
   </si>
   <si>
     <t>TC6</t>
@@ -140,7 +140,7 @@
     <t>Đã thực hiện gửi request đăng nhập không lưu phiên</t>
   </si>
   <si>
-    <t>16:30:50</t>
+    <t>16:48:11</t>
   </si>
   <si>
     <t>TC7</t>
@@ -152,7 +152,7 @@
     <t>username: '', password: ''</t>
   </si>
   <si>
-    <t>16:30:53</t>
+    <t>16:48:14</t>
   </si>
   <si>
     <t>TC8</t>
@@ -167,7 +167,7 @@
     <t>Hệ thống chặn truy cập, báo lỗi Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>16:30:56</t>
+    <t>16:48:18</t>
   </si>
   <si>
     <t>TC9</t>
@@ -179,7 +179,7 @@
     <t>username: 'admin\' --', password: 'password123'</t>
   </si>
   <si>
-    <t>16:30:58</t>
+    <t>16:48:21</t>
   </si>
   <si>
     <t>TC10</t>
@@ -197,7 +197,7 @@
     <t>Hệ thống xử lý an toàn: Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>16:31:01</t>
+    <t>16:48:29</t>
   </si>
   <si>
     <t>TC11</t>
@@ -215,7 +215,7 @@
     <t>Phản hồi hệ thống: Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>16:31:04</t>
+    <t>16:48:31</t>
   </si>
   <si>
     <t>TC12</t>
@@ -230,7 +230,7 @@
     <t>Báo lỗi Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>16:31:06</t>
+    <t>16:48:37</t>
   </si>
   <si>
     <t>TC13</t>
@@ -248,7 +248,7 @@
     <t>Thuộc tính type của ô mật khẩu là: password</t>
   </si>
   <si>
-    <t>16:31:09</t>
+    <t>16:48:39</t>
   </si>
   <si>
     <t>TC14</t>
@@ -266,7 +266,7 @@
     <t>Hệ thống chặn script thành công: Tài khoản hoặc mật khẩu không đúng.</t>
   </si>
   <si>
-    <t>16:31:11</t>
+    <t>16:48:41</t>
   </si>
   <si>
     <t>TC15</t>
@@ -281,7 +281,7 @@
     <t>Hệ thống xử lý chuỗi dài an toàn, không bị lỗi máy chủ (500)</t>
   </si>
   <si>
-    <t>16:31:14</t>
+    <t>16:48:44</t>
   </si>
   <si>
     <t>TC16</t>
@@ -299,7 +299,7 @@
     <t>Giá trị sau khi dán vào ô mật khẩu: 123456@utc</t>
   </si>
   <si>
-    <t>16:31:16</t>
+    <t>16:48:47</t>
   </si>
   <si>
     <t>TỔNG SỐ TEST CASE: 16</t>

</xml_diff>